<commit_message>
Model stats xlsx for plotting data
</commit_message>
<xml_diff>
--- a/data/JackNet_Stats.xlsx
+++ b/data/JackNet_Stats.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\jackr\Coral-TPU-Characterization\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0A70BBF-74A8-4CD4-81C7-4350F84A15FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8613F403-AFBE-4C70-8141-ED5E475E326A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="16220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -168,10 +168,10 @@
     <t>A075D08</t>
   </si>
   <si>
-    <t>A075D010</t>
-  </si>
-  <si>
     <t>Operation Count (M)</t>
+  </si>
+  <si>
+    <t>A075D01</t>
   </si>
 </sst>
 </file>
@@ -849,7 +849,7 @@
         <v>6</v>
       </c>
       <c r="G1" s="12" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="29.25" customHeight="1">
@@ -950,7 +950,7 @@
     </row>
     <row r="6" spans="1:9" ht="29.25" customHeight="1" thickBot="1">
       <c r="A6" s="13" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B6" s="14" t="s">
         <v>9</v>

</xml_diff>